<commit_message>
Apply AlphaForge patch: alpha_forge_v2_1_status_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Watchlist.xlsx
+++ b/AlphaForge_Watchlist.xlsx
@@ -1333,13 +1333,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>587993186304</v>
+        <v>587222351872</v>
       </c>
       <c r="G7" t="n">
-        <v>58.9</v>
+        <v>58.83</v>
       </c>
       <c r="H7" t="n">
-        <v>36.8</v>
+        <v>36.75</v>
       </c>
       <c r="I7" t="n">
         <v>29.71</v>
@@ -1363,16 +1363,16 @@
         <v>100</v>
       </c>
       <c r="P7" t="n">
-        <v>11.7</v>
+        <v>11.8</v>
       </c>
       <c r="Q7" t="n">
         <v>18.5</v>
       </c>
       <c r="R7" t="n">
-        <v>26.3</v>
+        <v>26.9</v>
       </c>
       <c r="S7" t="n">
-        <v>62.1</v>
+        <v>62.2</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1386,22 +1386,22 @@
       </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>1525.6</v>
+        <v>1523.6</v>
       </c>
       <c r="X7" t="n">
-        <v>16.85</v>
+        <v>16.7</v>
       </c>
       <c r="Y7" t="n">
-        <v>33.23</v>
+        <v>33.06</v>
       </c>
       <c r="Z7" t="n">
-        <v>60.89</v>
+        <v>60.68</v>
       </c>
       <c r="AA7" t="n">
-        <v>127.28</v>
+        <v>126.98</v>
       </c>
       <c r="AB7" t="n">
-        <v>32.49</v>
+        <v>32.43</v>
       </c>
       <c r="AC7" t="n">
         <v>38.1</v>
@@ -1413,10 +1413,10 @@
         <v>0.85</v>
       </c>
       <c r="AF7" t="n">
-        <v>1291.6401</v>
+        <v>1291.6001</v>
       </c>
       <c r="AG7" t="n">
-        <v>1052.303</v>
+        <v>1052.293</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         <v>18.5</v>
       </c>
       <c r="AL7" t="n">
-        <v>26.3</v>
+        <v>26.9</v>
       </c>
       <c r="AM7" t="n">
         <v>765</v>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v2_2_dashboard_status_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Watchlist.xlsx
+++ b/AlphaForge_Watchlist.xlsx
@@ -1333,13 +1333,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>587607769088</v>
+        <v>587838980096</v>
       </c>
       <c r="G7" t="n">
-        <v>58.86</v>
+        <v>58.89</v>
       </c>
       <c r="H7" t="n">
-        <v>36.77</v>
+        <v>36.79</v>
       </c>
       <c r="I7" t="n">
         <v>29.71</v>
@@ -1363,16 +1363,16 @@
         <v>100</v>
       </c>
       <c r="P7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="Q7" t="n">
         <v>18.5</v>
       </c>
       <c r="R7" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="S7" t="n">
-        <v>62.2</v>
+        <v>62.1</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1386,22 +1386,22 @@
       </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>1524.8</v>
+        <v>1525.2</v>
       </c>
       <c r="X7" t="n">
-        <v>16.79</v>
+        <v>16.82</v>
       </c>
       <c r="Y7" t="n">
-        <v>33.16</v>
+        <v>33.2</v>
       </c>
       <c r="Z7" t="n">
-        <v>60.81</v>
+        <v>60.85</v>
       </c>
       <c r="AA7" t="n">
-        <v>127.16</v>
+        <v>127.22</v>
       </c>
       <c r="AB7" t="n">
-        <v>32.47</v>
+        <v>32.48</v>
       </c>
       <c r="AC7" t="n">
         <v>38.1</v>
@@ -1413,10 +1413,10 @@
         <v>0.85</v>
       </c>
       <c r="AF7" t="n">
-        <v>1291.6241</v>
+        <v>1291.6321</v>
       </c>
       <c r="AG7" t="n">
-        <v>1052.299</v>
+        <v>1052.301</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
         <v>18.5</v>
       </c>
       <c r="AL7" t="n">
-        <v>26.5</v>
+        <v>26.4</v>
       </c>
       <c r="AM7" t="n">
         <v>765</v>

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v3_intelligence_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Watchlist.xlsx
+++ b/AlphaForge_Watchlist.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN10"/>
+  <dimension ref="A1:BC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -614,6 +614,81 @@
       </c>
       <c r="AN1" t="inlineStr">
         <is>
+          <t>Supporto 20D</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Supporto 60D</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Resistenza 20D</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Resistenza 60D</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Distanza MA50 %</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Distanza MA200 %</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Entry Zone</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>Risk Flag</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>Trigger Monitoraggio</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>Priority Score</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>Azione Suggerita</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>Scenario Base</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>Scenario Positivo</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>Scenario Negativo</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>Azione Pratica</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
           <t>Area</t>
         </is>
       </c>
@@ -750,7 +825,68 @@
       <c r="AM2" t="n">
         <v>751</v>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AN2" t="n">
+        <v>358.7757</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>273.3367</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>402.3797</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>402.3797</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>19.33</v>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>Medium-high risk</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW2" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>GOOGL: scenario base Buy Watchlist, score 80.2, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.1%.</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 402.38 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 273.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>USA / Internet</t>
         </is>
@@ -888,7 +1024,68 @@
       <c r="AM3" t="n">
         <v>751</v>
       </c>
-      <c r="AN3" t="inlineStr">
+      <c r="AN3" t="n">
+        <v>205.1</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>164.9777</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>235.4656</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>235.4656</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW3" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>NVDA: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 2.3%.</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 235.47 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 164.98 o peggioramento trend; rischio attuale: High risk.</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
         <is>
           <t>USA / Semiconductors</t>
         </is>
@@ -1026,7 +1223,68 @@
       <c r="AM4" t="n">
         <v>751</v>
       </c>
-      <c r="AN4" t="inlineStr">
+      <c r="AN4" t="n">
+        <v>292.68</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>246.403</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>315.2</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>315.2</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>Medium-high risk</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW4" t="n">
+        <v>70.59999999999999</v>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>AAPL: scenario base Accumulate Carefully, score 73.4, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 6.9%.</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 315.20 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 246.40 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
         <is>
           <t>USA / Technology</t>
         </is>
@@ -1162,7 +1420,68 @@
       <c r="AM5" t="n">
         <v>751</v>
       </c>
-      <c r="AN5" t="inlineStr">
+      <c r="AN5" t="n">
+        <v>245.22</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>199.34</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>274</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>274.99</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>-2.66</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>Medium-high risk</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW5" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>AMZN: scenario base Hold / Monitor, score 66.8, trend Constructive. Entry zone: Monitor / partial entry only. Distanza da MA50: -2.7%.</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 274.99 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 199.34 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
         <is>
           <t>USA / Consumer &amp; Cloud</t>
         </is>
@@ -1300,7 +1619,68 @@
       <c r="AM6" t="n">
         <v>751</v>
       </c>
-      <c r="AN6" t="inlineStr">
+      <c r="AN6" t="n">
+        <v>404.3343</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>355.9989</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>460.52</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>460.52</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>-9.31</v>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>Medium-high risk</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW6" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>MSFT: scenario base Hold / Monitor, score 65.5, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 0.8%.</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 460.52 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 356.00 o peggioramento trend; rischio attuale: Medium-high risk.</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
         <is>
           <t>USA / Technology</t>
         </is>
@@ -1333,13 +1713,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>587607769088</v>
+        <v>590305689600</v>
       </c>
       <c r="G7" t="n">
-        <v>58.86</v>
+        <v>59.14</v>
       </c>
       <c r="H7" t="n">
-        <v>36.77</v>
+        <v>36.94</v>
       </c>
       <c r="I7" t="n">
         <v>29.71</v>
@@ -1363,16 +1743,16 @@
         <v>100</v>
       </c>
       <c r="P7" t="n">
-        <v>11.8</v>
+        <v>11.5</v>
       </c>
       <c r="Q7" t="n">
         <v>18.5</v>
       </c>
       <c r="R7" t="n">
-        <v>26.6</v>
+        <v>24.5</v>
       </c>
       <c r="S7" t="n">
-        <v>62.2</v>
+        <v>61.9</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1386,37 +1766,37 @@
       </c>
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="n">
-        <v>1524.6</v>
+        <v>1531.6</v>
       </c>
       <c r="X7" t="n">
-        <v>16.77</v>
+        <v>17.31</v>
       </c>
       <c r="Y7" t="n">
-        <v>33.14</v>
+        <v>33.76</v>
       </c>
       <c r="Z7" t="n">
-        <v>60.78</v>
+        <v>61.52</v>
       </c>
       <c r="AA7" t="n">
-        <v>127.13</v>
+        <v>128.18</v>
       </c>
       <c r="AB7" t="n">
-        <v>32.46</v>
+        <v>32.66</v>
       </c>
       <c r="AC7" t="n">
-        <v>38.1</v>
+        <v>38.11</v>
       </c>
       <c r="AD7" t="n">
         <v>-44.77</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="AF7" t="n">
-        <v>1291.6201</v>
+        <v>1291.7601</v>
       </c>
       <c r="AG7" t="n">
-        <v>1052.298</v>
+        <v>1052.333</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
@@ -1433,12 +1813,73 @@
         <v>18.5</v>
       </c>
       <c r="AL7" t="n">
-        <v>26.6</v>
+        <v>24.5</v>
       </c>
       <c r="AM7" t="n">
         <v>765</v>
       </c>
-      <c r="AN7" t="inlineStr">
+      <c r="AN7" t="n">
+        <v>1249</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>1109.5466</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>1531.6</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>1531.6</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>18.57</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>45.54</v>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>Extended - wait pullback</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>prezzo 18.6% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+        </is>
+      </c>
+      <c r="AW7" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>ASML.AS: scenario base Hold / Monitor, score 61.9, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.6%.</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 1531.60 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 1109.55 o peggioramento trend; rischio attuale: High risk.</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
         <is>
           <t>Europe / Semiconductors</t>
         </is>
@@ -1576,7 +2017,68 @@
       <c r="AM8" t="n">
         <v>751</v>
       </c>
-      <c r="AN8" t="inlineStr">
+      <c r="AN8" t="n">
+        <v>585.39</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>525.72</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>635.29</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>688.55</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>-5.62</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>-11.43</v>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Wait for trend repair</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>prezzo 5.6% sotto MA50: attendere recupero</t>
+        </is>
+      </c>
+      <c r="AW8" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>META: scenario base Hold / Monitor, score 59.4, trend Weak. Entry zone: Wait for trend repair. Distanza da MA50: -5.6%.</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 688.55 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 525.72 o peggioramento trend; rischio attuale: High risk.</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
         <is>
           <t>USA / Social &amp; AI</t>
         </is>
@@ -1712,7 +2214,68 @@
       <c r="AM9" t="n">
         <v>751</v>
       </c>
-      <c r="AN9" t="inlineStr">
+      <c r="AN9" t="n">
+        <v>391</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>343.25</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>445.27</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>445.27</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>-1.35</v>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Monitor / partial entry only</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>High risk</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>prezzo vicino a MA50: monitorare conferma</t>
+        </is>
+      </c>
+      <c r="AW9" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>Ridurre size / solo monitoraggio</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>TSLA: scenario base High Risk, score 41.3, trend Recovery. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.3%.</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area 445.27 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area 343.25 o peggioramento trend; rischio attuale: High risk.</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
         <is>
           <t>USA / EV</t>
         </is>
@@ -1810,7 +2373,56 @@
       <c r="AM10" t="n">
         <v>0</v>
       </c>
-      <c r="AN10" t="inlineStr">
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>No Data</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>No Data</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>Dati prezzo insufficienti.</t>
+        </is>
+      </c>
+      <c r="AW10" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Evitare per ora</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>STM.MI: scenario base Avoid for Now, score 38.5, trend No Data. Entry zone: No Data. Distanza da MA50: n/d.</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>Scenario positivo: conferma sopra area n/d con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>Scenario negativo: perdita area n/d o peggioramento trend; rischio attuale: No Data.</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>Azione pratica: non trasformare lo score in ordine automatico; usa watchlist, alert prezzo, controllo news/trimestrali e dimensione posizione.</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
         <is>
           <t>Italy / Semiconductors</t>
         </is>

</xml_diff>